<commit_message>
Add offline survey details data caching
</commit_message>
<xml_diff>
--- a/data/mill_return.xlsx
+++ b/data/mill_return.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2905"/>
+  <dimension ref="A1:G2919"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85499,6 +85499,440 @@
         </is>
       </c>
     </row>
+    <row r="2906">
+      <c r="A2906" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B2906" t="inlineStr">
+        <is>
+          <t>5306</t>
+        </is>
+      </c>
+      <c r="C2906" t="inlineStr">
+        <is>
+          <t>R579</t>
+        </is>
+      </c>
+      <c r="D2906" t="n">
+        <v>16</v>
+      </c>
+      <c r="E2906" t="n">
+        <v>147.15</v>
+      </c>
+      <c r="F2906" t="n">
+        <v>9.196999999999999</v>
+      </c>
+      <c r="G2906" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2907">
+      <c r="A2907" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B2907" t="inlineStr">
+        <is>
+          <t>5306</t>
+        </is>
+      </c>
+      <c r="C2907" t="inlineStr">
+        <is>
+          <t>R579</t>
+        </is>
+      </c>
+      <c r="D2907" t="n">
+        <v>81</v>
+      </c>
+      <c r="E2907" t="n">
+        <v>692.7</v>
+      </c>
+      <c r="F2907" t="n">
+        <v>8.552</v>
+      </c>
+      <c r="G2907" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2908">
+      <c r="A2908" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B2908" t="inlineStr">
+        <is>
+          <t>5217</t>
+        </is>
+      </c>
+      <c r="C2908" t="inlineStr">
+        <is>
+          <t>R579</t>
+        </is>
+      </c>
+      <c r="D2908" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2908" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="F2908" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="G2908" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2909">
+      <c r="A2909" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B2909" t="inlineStr">
+        <is>
+          <t>4212</t>
+        </is>
+      </c>
+      <c r="C2909" t="inlineStr">
+        <is>
+          <t>97F1692</t>
+        </is>
+      </c>
+      <c r="D2909" t="n">
+        <v>112</v>
+      </c>
+      <c r="E2909" t="n">
+        <v>669.59</v>
+      </c>
+      <c r="F2909" t="n">
+        <v>5.978</v>
+      </c>
+      <c r="G2909" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2910">
+      <c r="A2910" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B2910" t="inlineStr">
+        <is>
+          <t>5440</t>
+        </is>
+      </c>
+      <c r="C2910" t="inlineStr">
+        <is>
+          <t>R579</t>
+        </is>
+      </c>
+      <c r="D2910" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2910" t="n">
+        <v>15.58</v>
+      </c>
+      <c r="F2910" t="n">
+        <v>5.193</v>
+      </c>
+      <c r="G2910" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2911">
+      <c r="A2911" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B2911" t="inlineStr">
+        <is>
+          <t>4212</t>
+        </is>
+      </c>
+      <c r="C2911" t="inlineStr">
+        <is>
+          <t>97F1692</t>
+        </is>
+      </c>
+      <c r="D2911" t="n">
+        <v>36</v>
+      </c>
+      <c r="E2911" t="n">
+        <v>215.53</v>
+      </c>
+      <c r="F2911" t="n">
+        <v>5.987</v>
+      </c>
+      <c r="G2911" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2912">
+      <c r="A2912" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B2912" t="inlineStr">
+        <is>
+          <t>3107</t>
+        </is>
+      </c>
+      <c r="C2912" t="inlineStr">
+        <is>
+          <t>R579</t>
+        </is>
+      </c>
+      <c r="D2912" t="n">
+        <v>72</v>
+      </c>
+      <c r="E2912" t="n">
+        <v>504.02</v>
+      </c>
+      <c r="F2912" t="n">
+        <v>7</v>
+      </c>
+      <c r="G2912" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2913">
+      <c r="A2913" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B2913" t="inlineStr">
+        <is>
+          <t>5306</t>
+        </is>
+      </c>
+      <c r="C2913" t="inlineStr">
+        <is>
+          <t>R579</t>
+        </is>
+      </c>
+      <c r="D2913" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2913" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="F2913" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="G2913" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2914">
+      <c r="A2914" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B2914" t="inlineStr">
+        <is>
+          <t>5410</t>
+        </is>
+      </c>
+      <c r="C2914" t="inlineStr">
+        <is>
+          <t>R579</t>
+        </is>
+      </c>
+      <c r="D2914" t="n">
+        <v>61</v>
+      </c>
+      <c r="E2914" t="n">
+        <v>438.84</v>
+      </c>
+      <c r="F2914" t="n">
+        <v>7.194</v>
+      </c>
+      <c r="G2914" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2915">
+      <c r="A2915" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B2915" t="inlineStr">
+        <is>
+          <t>3107</t>
+        </is>
+      </c>
+      <c r="C2915" t="inlineStr">
+        <is>
+          <t>R579</t>
+        </is>
+      </c>
+      <c r="D2915" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2915" t="n">
+        <v>43.29</v>
+      </c>
+      <c r="F2915" t="n">
+        <v>7.215</v>
+      </c>
+      <c r="G2915" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2916">
+      <c r="A2916" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B2916" t="inlineStr">
+        <is>
+          <t>5205</t>
+        </is>
+      </c>
+      <c r="C2916" t="inlineStr">
+        <is>
+          <t>R579</t>
+        </is>
+      </c>
+      <c r="D2916" t="n">
+        <v>89</v>
+      </c>
+      <c r="E2916" t="n">
+        <v>699.54</v>
+      </c>
+      <c r="F2916" t="n">
+        <v>7.86</v>
+      </c>
+      <c r="G2916" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2917">
+      <c r="A2917" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B2917" t="inlineStr">
+        <is>
+          <t>1213</t>
+        </is>
+      </c>
+      <c r="C2917" t="inlineStr">
+        <is>
+          <t>R579</t>
+        </is>
+      </c>
+      <c r="D2917" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2917" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="F2917" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="G2917" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2918">
+      <c r="A2918" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B2918" t="inlineStr">
+        <is>
+          <t>5702</t>
+        </is>
+      </c>
+      <c r="C2918" t="inlineStr">
+        <is>
+          <t>R579</t>
+        </is>
+      </c>
+      <c r="D2918" t="n">
+        <v>82</v>
+      </c>
+      <c r="E2918" t="n">
+        <v>585.76</v>
+      </c>
+      <c r="F2918" t="n">
+        <v>7.143</v>
+      </c>
+      <c r="G2918" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2919">
+      <c r="A2919" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B2919" t="inlineStr">
+        <is>
+          <t>5306</t>
+        </is>
+      </c>
+      <c r="C2919" t="inlineStr">
+        <is>
+          <t>R579</t>
+        </is>
+      </c>
+      <c r="D2919" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2919" t="n">
+        <v>27.22</v>
+      </c>
+      <c r="F2919" t="n">
+        <v>6.805</v>
+      </c>
+      <c r="G2919" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>